<commit_message>
feat(rules): G01-P7-M11 execute exact event observations
</commit_message>
<xml_diff>
--- a/config/generated/templates/EventFilter.xlsx
+++ b/config/generated/templates/EventFilter.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="44">
   <si>
     <t>@table</t>
   </si>
@@ -43,7 +43,7 @@
     <t>@schema</t>
   </si>
   <si>
-    <t>8adac0f1c78cd386</t>
+    <t>647b6f13916c7a3d</t>
   </si>
   <si>
     <t>#name</t>
@@ -82,6 +82,12 @@
     <t>damage_class</t>
   </si>
   <si>
+    <t>resource_kind</t>
+  </si>
+  <si>
+    <t>character_resource_key</t>
+  </si>
+  <si>
     <t>cause_ancestry</t>
   </si>
   <si>
@@ -118,6 +124,9 @@
     <t>optional&lt;enum&lt;DamageClass&gt;&gt;</t>
   </si>
   <si>
+    <t>optional&lt;enum&lt;ResourceKind&gt;&gt;</t>
+  </si>
+  <si>
     <t>enum&lt;CauseAncestry&gt;</t>
   </si>
   <si>
@@ -131,6 +140,9 @@
   </si>
   <si>
     <t>length=1..160</t>
+  </si>
+  <si>
+    <t>length=1..120</t>
   </si>
   <si>
     <t>#desc</t>
@@ -550,7 +562,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -561,10 +573,12 @@
     <col min="11" max="11" width="16.7109375" style="5" customWidth="1"/>
     <col min="12" max="12" width="29.7109375" style="5" customWidth="1"/>
     <col min="13" max="13" width="27.7109375" style="5" customWidth="1"/>
-    <col min="14" max="14" width="19.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="28.7109375" style="5" customWidth="1"/>
+    <col min="15" max="15" width="22.7109375" style="5" customWidth="1"/>
+    <col min="16" max="16" width="19.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -596,7 +610,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="24" customHeight="1">
+    <row r="2" spans="1:16" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -639,10 +653,16 @@
       <c r="N2" s="3" t="s">
         <v>22</v>
       </c>
+      <c r="O2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:16">
       <c r="A3" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>5</v>
@@ -683,54 +703,66 @@
       <c r="N3" s="5" t="s">
         <v>22</v>
       </c>
+      <c r="O3" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:16">
       <c r="A4" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O4" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="N4" s="5" t="s">
-        <v>34</v>
+      <c r="P4" s="5" t="s">
+        <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:16">
       <c r="A5" s="4" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>7</v>
@@ -771,16 +803,22 @@
       <c r="N5" s="5" t="s">
         <v>7</v>
       </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:16">
       <c r="A6" s="4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
@@ -793,10 +831,14 @@
       <c r="L6" s="5"/>
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
+      <c r="O6" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="P6" s="5"/>
     </row>
-    <row r="7" spans="1:14" ht="42" customHeight="1">
+    <row r="7" spans="1:16" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -811,9 +853,11 @@
       <c r="L7" s="6"/>
       <c r="M7" s="6"/>
       <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
     </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="7">
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
@@ -830,7 +874,10 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Ordinary, Dot, Break, SuperBreak, Additional, Joint, Elation, TrueDamage" promptTitle="DamageClass enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
       <formula1>"Ordinary,Dot,Break,SuperBreak,Additional,Joint,Elation,TrueDamage"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Any, RootCommand, DirectParent, SameAction, SamePhase, SameHit" promptTitle="CauseAncestry enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Energy, SkillPoints, Hp, CharacterResource, TeamResource" promptTitle="ResourceKind enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
+      <formula1>"Energy,SkillPoints,Hp,CharacterResource,TeamResource"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Any, RootCommand, DirectParent, SameAction, SamePhase, SameHit" promptTitle="CauseAncestry enum" prompt="Select a value from the dropdown." sqref="P8:P1007">
       <formula1>"Any,RootCommand,DirectParent,SameAction,SamePhase,SameHit"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>